<commit_message>
Finalising KO run (in progress)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013o7QrhEUYPhCLzn4AyzH1S
</commit_message>
<xml_diff>
--- a/runs/KO/2026-10-13/bear/scratch/audit_erp_fernandez_5p5/dcf.xlsx
+++ b/runs/KO/2026-10-13/bear/scratch/audit_erp_fernandez_5p5/dcf.xlsx
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0.04759004187363834</v>
+        <v>0.04759004187363835</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -972,7 +972,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>0.03</v>
@@ -1018,7 +1018,7 @@
         <v/>
       </c>
       <c r="I3" s="4" t="n">
-        <v>52862.02214222582</v>
+        <v>52363.32382012936</v>
       </c>
     </row>
     <row r="4">
@@ -1075,7 +1075,7 @@
         <v/>
       </c>
       <c r="I5" s="4" t="n">
-        <v>17545.43376922617</v>
+        <v>17379.91080913914</v>
       </c>
     </row>
     <row r="6">
@@ -1240,7 +1240,7 @@
         <v/>
       </c>
       <c r="I11" s="4" t="n">
-        <v>12634.26193579465</v>
+        <v>12515.07078545696</v>
       </c>
     </row>
     <row r="12">
@@ -1351,7 +1351,7 @@
         <v/>
       </c>
       <c r="I15" s="4" t="n">
-        <v>8832.022666001165</v>
+        <v>8748.701697453986</v>
       </c>
     </row>
     <row r="16">
@@ -1419,7 +1419,7 @@
         <v/>
       </c>
       <c r="C20" s="4" t="n">
-        <v>49054.07875876826</v>
+        <v>48550.10563511542</v>
       </c>
     </row>
     <row r="21">
@@ -1433,7 +1433,7 @@
         <v/>
       </c>
       <c r="C21" s="4" t="n">
-        <v>12643.43452336848</v>
+        <v>12524.15683918576</v>
       </c>
     </row>
     <row r="22">
@@ -1447,7 +1447,7 @@
         <v/>
       </c>
       <c r="C22" s="4" t="n">
-        <v>201288.4587563877</v>
+        <v>199389.5110322709</v>
       </c>
     </row>
     <row r="23">
@@ -1461,7 +1461,7 @@
         <v/>
       </c>
       <c r="C23" s="4" t="n">
-        <v>140711.3640017343</v>
+        <v>139383.8983036048</v>
       </c>
     </row>
     <row r="24">
@@ -1475,7 +1475,7 @@
         <v/>
       </c>
       <c r="C24" s="4" t="n">
-        <v>189765.4427605026</v>
+        <v>187934.0039387202</v>
       </c>
     </row>
     <row r="25">
@@ -1503,7 +1503,7 @@
         <v/>
       </c>
       <c r="C26" s="4" t="n">
-        <v>190176.9427605026</v>
+        <v>188345.5039387202</v>
       </c>
     </row>
     <row r="27">
@@ -1517,7 +1517,7 @@
         <v/>
       </c>
       <c r="C27" s="4" t="n">
-        <v>193361.5673571504</v>
+        <v>191408.2474637605</v>
       </c>
     </row>
     <row r="28">
@@ -1531,7 +1531,7 @@
         <v/>
       </c>
       <c r="C28" s="4" t="n">
-        <v>44.94690082685969</v>
+        <v>44.49285157223629</v>
       </c>
     </row>
     <row r="29">
@@ -1545,7 +1545,7 @@
         <v/>
       </c>
       <c r="C29" s="6" t="n">
-        <v>-0.5012549994</v>
+        <v>-0.5062932731999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>